<commit_message>
Improve home and My Work UX, persist Gmail, and expand survey ops.
Home page redesign, Gmail auto-connect on Google sign-in with DB-backed tokens, My Work email panel, GPS/photo/audio capture in Studio, survey link agent, PM stage sorting/import updates, and removal of manual Excel import UI from Operations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/assets/import/project_import_master.xlsx
+++ b/backend/assets/import/project_import_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sunilmukkath/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sunilmukkath/Lime Survey ET DB/RETLS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27EEA370-DED2-A34D-8925-E417EC39FD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FDF371-CE35-7F49-84A9-0DB312510E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="600" windowWidth="25440" windowHeight="14760" xr2:uid="{A9BAE5F9-AA28-DD4E-B912-0DDEBD9E5A6E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="473">
   <si>
     <t>project_name</t>
   </si>
@@ -1455,6 +1455,9 @@
   </si>
   <si>
     <t>Project_Value_INR</t>
+  </si>
+  <si>
+    <t>Delivered</t>
   </si>
 </sst>
 </file>
@@ -1892,6 +1895,9 @@
       <c r="E2" t="s">
         <v>204</v>
       </c>
+      <c r="J2" t="s">
+        <v>472</v>
+      </c>
       <c r="K2" t="s">
         <v>465</v>
       </c>
@@ -1915,6 +1921,9 @@
       <c r="E3" t="s">
         <v>206</v>
       </c>
+      <c r="J3" t="s">
+        <v>472</v>
+      </c>
       <c r="K3" t="s">
         <v>465</v>
       </c>
@@ -1938,6 +1947,9 @@
       <c r="E4" t="s">
         <v>208</v>
       </c>
+      <c r="J4" t="s">
+        <v>472</v>
+      </c>
       <c r="K4" t="s">
         <v>465</v>
       </c>
@@ -1961,6 +1973,9 @@
       <c r="E5" t="s">
         <v>210</v>
       </c>
+      <c r="J5" t="s">
+        <v>472</v>
+      </c>
       <c r="K5" t="s">
         <v>466</v>
       </c>
@@ -1984,6 +1999,9 @@
       <c r="E6" t="s">
         <v>212</v>
       </c>
+      <c r="J6" t="s">
+        <v>472</v>
+      </c>
       <c r="K6" t="s">
         <v>465</v>
       </c>
@@ -2007,6 +2025,9 @@
       <c r="E7" t="s">
         <v>214</v>
       </c>
+      <c r="J7" t="s">
+        <v>472</v>
+      </c>
       <c r="K7" t="s">
         <v>465</v>
       </c>
@@ -2030,6 +2051,9 @@
       <c r="E8" t="s">
         <v>216</v>
       </c>
+      <c r="J8" t="s">
+        <v>472</v>
+      </c>
       <c r="K8" t="s">
         <v>465</v>
       </c>
@@ -2053,6 +2077,9 @@
       <c r="E9" t="s">
         <v>218</v>
       </c>
+      <c r="J9" t="s">
+        <v>472</v>
+      </c>
       <c r="K9" t="s">
         <v>465</v>
       </c>
@@ -2076,6 +2103,9 @@
       <c r="E10" t="s">
         <v>220</v>
       </c>
+      <c r="J10" t="s">
+        <v>472</v>
+      </c>
       <c r="K10" t="s">
         <v>467</v>
       </c>
@@ -2099,6 +2129,9 @@
       <c r="E11" t="s">
         <v>222</v>
       </c>
+      <c r="J11" t="s">
+        <v>472</v>
+      </c>
       <c r="K11" t="s">
         <v>467</v>
       </c>
@@ -2122,6 +2155,9 @@
       <c r="E12" t="s">
         <v>225</v>
       </c>
+      <c r="J12" t="s">
+        <v>472</v>
+      </c>
       <c r="K12" t="s">
         <v>465</v>
       </c>
@@ -2145,6 +2181,9 @@
       <c r="E13" t="s">
         <v>226</v>
       </c>
+      <c r="J13" t="s">
+        <v>472</v>
+      </c>
       <c r="K13" t="s">
         <v>465</v>
       </c>
@@ -2168,6 +2207,9 @@
       <c r="E14" t="s">
         <v>228</v>
       </c>
+      <c r="J14" t="s">
+        <v>472</v>
+      </c>
       <c r="K14" t="s">
         <v>467</v>
       </c>
@@ -2191,6 +2233,9 @@
       <c r="E15" t="s">
         <v>230</v>
       </c>
+      <c r="J15" t="s">
+        <v>472</v>
+      </c>
       <c r="K15" t="s">
         <v>465</v>
       </c>
@@ -2214,6 +2259,9 @@
       <c r="E16" t="s">
         <v>232</v>
       </c>
+      <c r="J16" t="s">
+        <v>472</v>
+      </c>
       <c r="K16" t="s">
         <v>465</v>
       </c>
@@ -2237,6 +2285,9 @@
       <c r="E17" t="s">
         <v>233</v>
       </c>
+      <c r="J17" t="s">
+        <v>472</v>
+      </c>
       <c r="K17" t="s">
         <v>468</v>
       </c>
@@ -2260,6 +2311,9 @@
       <c r="E18" t="s">
         <v>235</v>
       </c>
+      <c r="J18" t="s">
+        <v>472</v>
+      </c>
       <c r="K18" t="s">
         <v>468</v>
       </c>
@@ -2283,6 +2337,9 @@
       <c r="E19" t="s">
         <v>236</v>
       </c>
+      <c r="J19" t="s">
+        <v>472</v>
+      </c>
       <c r="K19" t="s">
         <v>465</v>
       </c>
@@ -2306,6 +2363,9 @@
       <c r="E20" t="s">
         <v>237</v>
       </c>
+      <c r="J20" t="s">
+        <v>472</v>
+      </c>
       <c r="K20" t="s">
         <v>467</v>
       </c>
@@ -2329,6 +2389,9 @@
       <c r="E21" t="s">
         <v>239</v>
       </c>
+      <c r="J21" t="s">
+        <v>472</v>
+      </c>
       <c r="K21" t="s">
         <v>465</v>
       </c>
@@ -2352,6 +2415,9 @@
       <c r="E22" t="s">
         <v>241</v>
       </c>
+      <c r="J22" t="s">
+        <v>472</v>
+      </c>
       <c r="K22" t="s">
         <v>468</v>
       </c>
@@ -2375,6 +2441,9 @@
       <c r="E23" t="s">
         <v>243</v>
       </c>
+      <c r="J23" t="s">
+        <v>472</v>
+      </c>
       <c r="K23" t="s">
         <v>465</v>
       </c>
@@ -2398,6 +2467,9 @@
       <c r="E24" t="s">
         <v>245</v>
       </c>
+      <c r="J24" t="s">
+        <v>472</v>
+      </c>
       <c r="K24" t="s">
         <v>468</v>
       </c>
@@ -2421,6 +2493,9 @@
       <c r="E25" t="s">
         <v>246</v>
       </c>
+      <c r="J25" t="s">
+        <v>472</v>
+      </c>
       <c r="K25" t="s">
         <v>465</v>
       </c>
@@ -2444,6 +2519,9 @@
       <c r="E26" t="s">
         <v>248</v>
       </c>
+      <c r="J26" t="s">
+        <v>472</v>
+      </c>
       <c r="K26" t="s">
         <v>465</v>
       </c>
@@ -2467,6 +2545,9 @@
       <c r="E27" t="s">
         <v>250</v>
       </c>
+      <c r="J27" t="s">
+        <v>472</v>
+      </c>
       <c r="K27" t="s">
         <v>465</v>
       </c>
@@ -2490,6 +2571,9 @@
       <c r="E28" t="s">
         <v>252</v>
       </c>
+      <c r="J28" t="s">
+        <v>472</v>
+      </c>
       <c r="K28" t="s">
         <v>467</v>
       </c>
@@ -2513,6 +2597,9 @@
       <c r="E29" t="s">
         <v>254</v>
       </c>
+      <c r="J29" t="s">
+        <v>472</v>
+      </c>
       <c r="K29" t="s">
         <v>465</v>
       </c>
@@ -2536,6 +2623,9 @@
       <c r="E30" t="s">
         <v>255</v>
       </c>
+      <c r="J30" t="s">
+        <v>472</v>
+      </c>
       <c r="K30" t="s">
         <v>465</v>
       </c>
@@ -2559,6 +2649,9 @@
       <c r="E31" t="s">
         <v>256</v>
       </c>
+      <c r="J31" t="s">
+        <v>472</v>
+      </c>
       <c r="K31" t="s">
         <v>465</v>
       </c>
@@ -2582,6 +2675,9 @@
       <c r="E32" t="s">
         <v>257</v>
       </c>
+      <c r="J32" t="s">
+        <v>472</v>
+      </c>
       <c r="K32" t="s">
         <v>465</v>
       </c>
@@ -2605,6 +2701,9 @@
       <c r="E33" t="s">
         <v>258</v>
       </c>
+      <c r="J33" t="s">
+        <v>472</v>
+      </c>
       <c r="K33" t="s">
         <v>465</v>
       </c>
@@ -2628,6 +2727,9 @@
       <c r="E34" t="s">
         <v>260</v>
       </c>
+      <c r="J34" t="s">
+        <v>472</v>
+      </c>
       <c r="K34" t="s">
         <v>465</v>
       </c>
@@ -2651,6 +2753,9 @@
       <c r="E35" t="s">
         <v>262</v>
       </c>
+      <c r="J35" t="s">
+        <v>472</v>
+      </c>
       <c r="K35" t="s">
         <v>465</v>
       </c>
@@ -2674,6 +2779,9 @@
       <c r="E36" t="s">
         <v>264</v>
       </c>
+      <c r="J36" t="s">
+        <v>472</v>
+      </c>
       <c r="K36" t="s">
         <v>465</v>
       </c>
@@ -2697,6 +2805,9 @@
       <c r="E37" t="s">
         <v>266</v>
       </c>
+      <c r="J37" t="s">
+        <v>472</v>
+      </c>
       <c r="K37" t="s">
         <v>467</v>
       </c>
@@ -2720,6 +2831,9 @@
       <c r="E38" t="s">
         <v>268</v>
       </c>
+      <c r="J38" t="s">
+        <v>472</v>
+      </c>
       <c r="K38" t="s">
         <v>465</v>
       </c>
@@ -2743,6 +2857,9 @@
       <c r="E39" t="s">
         <v>269</v>
       </c>
+      <c r="J39" t="s">
+        <v>472</v>
+      </c>
       <c r="K39" t="s">
         <v>465</v>
       </c>
@@ -2766,6 +2883,9 @@
       <c r="E40" t="s">
         <v>271</v>
       </c>
+      <c r="J40" t="s">
+        <v>472</v>
+      </c>
       <c r="K40" t="s">
         <v>465</v>
       </c>
@@ -2789,6 +2909,9 @@
       <c r="E41" t="s">
         <v>273</v>
       </c>
+      <c r="J41" t="s">
+        <v>472</v>
+      </c>
       <c r="K41" t="s">
         <v>467</v>
       </c>
@@ -2812,6 +2935,9 @@
       <c r="E42" t="s">
         <v>274</v>
       </c>
+      <c r="J42" t="s">
+        <v>472</v>
+      </c>
       <c r="K42" t="s">
         <v>467</v>
       </c>
@@ -2835,6 +2961,9 @@
       <c r="E43" t="s">
         <v>275</v>
       </c>
+      <c r="J43" t="s">
+        <v>472</v>
+      </c>
       <c r="K43" t="s">
         <v>465</v>
       </c>
@@ -2858,6 +2987,9 @@
       <c r="E44" t="s">
         <v>277</v>
       </c>
+      <c r="J44" t="s">
+        <v>472</v>
+      </c>
       <c r="K44" t="s">
         <v>467</v>
       </c>
@@ -2881,6 +3013,9 @@
       <c r="E45" t="s">
         <v>278</v>
       </c>
+      <c r="J45" t="s">
+        <v>472</v>
+      </c>
       <c r="K45" t="s">
         <v>467</v>
       </c>
@@ -2904,6 +3039,9 @@
       <c r="E46" t="s">
         <v>280</v>
       </c>
+      <c r="J46" t="s">
+        <v>472</v>
+      </c>
       <c r="K46" t="s">
         <v>465</v>
       </c>
@@ -2927,6 +3065,9 @@
       <c r="E47" t="s">
         <v>281</v>
       </c>
+      <c r="J47" t="s">
+        <v>472</v>
+      </c>
       <c r="K47" t="s">
         <v>467</v>
       </c>
@@ -2950,6 +3091,9 @@
       <c r="E48" t="s">
         <v>282</v>
       </c>
+      <c r="J48" t="s">
+        <v>472</v>
+      </c>
       <c r="K48" t="s">
         <v>465</v>
       </c>
@@ -2973,6 +3117,9 @@
       <c r="E49" t="s">
         <v>283</v>
       </c>
+      <c r="J49" t="s">
+        <v>472</v>
+      </c>
       <c r="K49" t="s">
         <v>465</v>
       </c>
@@ -2996,6 +3143,9 @@
       <c r="E50" t="s">
         <v>285</v>
       </c>
+      <c r="J50" t="s">
+        <v>472</v>
+      </c>
       <c r="K50" t="s">
         <v>465</v>
       </c>
@@ -3019,6 +3169,9 @@
       <c r="E51" t="s">
         <v>286</v>
       </c>
+      <c r="J51" t="s">
+        <v>472</v>
+      </c>
       <c r="K51" t="s">
         <v>465</v>
       </c>
@@ -3042,6 +3195,9 @@
       <c r="E52" t="s">
         <v>288</v>
       </c>
+      <c r="J52" t="s">
+        <v>472</v>
+      </c>
       <c r="K52" t="s">
         <v>465</v>
       </c>
@@ -3065,6 +3221,9 @@
       <c r="E53" t="s">
         <v>289</v>
       </c>
+      <c r="J53" t="s">
+        <v>472</v>
+      </c>
       <c r="K53" t="s">
         <v>467</v>
       </c>
@@ -3088,6 +3247,9 @@
       <c r="E54" t="s">
         <v>291</v>
       </c>
+      <c r="J54" t="s">
+        <v>472</v>
+      </c>
       <c r="K54" t="s">
         <v>465</v>
       </c>
@@ -3111,6 +3273,9 @@
       <c r="E55" t="s">
         <v>292</v>
       </c>
+      <c r="J55" t="s">
+        <v>472</v>
+      </c>
       <c r="K55" t="s">
         <v>465</v>
       </c>
@@ -3134,6 +3299,9 @@
       <c r="E56" t="s">
         <v>294</v>
       </c>
+      <c r="J56" t="s">
+        <v>472</v>
+      </c>
       <c r="K56" t="s">
         <v>465</v>
       </c>
@@ -3157,6 +3325,9 @@
       <c r="E57" t="s">
         <v>295</v>
       </c>
+      <c r="J57" t="s">
+        <v>472</v>
+      </c>
       <c r="K57" t="s">
         <v>465</v>
       </c>
@@ -3180,6 +3351,9 @@
       <c r="E58" t="s">
         <v>297</v>
       </c>
+      <c r="J58" t="s">
+        <v>472</v>
+      </c>
       <c r="K58" t="s">
         <v>467</v>
       </c>
@@ -3203,6 +3377,9 @@
       <c r="E59" t="s">
         <v>298</v>
       </c>
+      <c r="J59" t="s">
+        <v>472</v>
+      </c>
       <c r="K59" t="s">
         <v>465</v>
       </c>
@@ -3226,6 +3403,9 @@
       <c r="E60" t="s">
         <v>299</v>
       </c>
+      <c r="J60" t="s">
+        <v>472</v>
+      </c>
       <c r="K60" t="s">
         <v>465</v>
       </c>
@@ -3249,6 +3429,9 @@
       <c r="E61" t="s">
         <v>300</v>
       </c>
+      <c r="J61" t="s">
+        <v>472</v>
+      </c>
       <c r="K61" t="s">
         <v>465</v>
       </c>
@@ -3272,6 +3455,9 @@
       <c r="E62" t="s">
         <v>301</v>
       </c>
+      <c r="J62" t="s">
+        <v>472</v>
+      </c>
       <c r="K62" t="s">
         <v>467</v>
       </c>
@@ -3295,6 +3481,9 @@
       <c r="E63" t="s">
         <v>303</v>
       </c>
+      <c r="J63" t="s">
+        <v>472</v>
+      </c>
       <c r="K63" t="s">
         <v>465</v>
       </c>
@@ -3318,6 +3507,9 @@
       <c r="E64" t="s">
         <v>304</v>
       </c>
+      <c r="J64" t="s">
+        <v>472</v>
+      </c>
       <c r="K64" t="s">
         <v>465</v>
       </c>
@@ -3341,6 +3533,9 @@
       <c r="E65" t="s">
         <v>306</v>
       </c>
+      <c r="J65" t="s">
+        <v>472</v>
+      </c>
       <c r="K65" t="s">
         <v>465</v>
       </c>
@@ -3364,6 +3559,9 @@
       <c r="E66" t="s">
         <v>307</v>
       </c>
+      <c r="J66" t="s">
+        <v>472</v>
+      </c>
       <c r="K66" t="s">
         <v>465</v>
       </c>
@@ -3387,6 +3585,9 @@
       <c r="E67" t="s">
         <v>308</v>
       </c>
+      <c r="J67" t="s">
+        <v>472</v>
+      </c>
       <c r="K67" t="s">
         <v>465</v>
       </c>
@@ -3410,6 +3611,9 @@
       <c r="E68" t="s">
         <v>309</v>
       </c>
+      <c r="J68" t="s">
+        <v>472</v>
+      </c>
       <c r="K68" t="s">
         <v>467</v>
       </c>
@@ -3433,6 +3637,9 @@
       <c r="E69" t="s">
         <v>310</v>
       </c>
+      <c r="J69" t="s">
+        <v>472</v>
+      </c>
       <c r="K69" t="s">
         <v>468</v>
       </c>
@@ -3456,6 +3663,9 @@
       <c r="E70" t="s">
         <v>311</v>
       </c>
+      <c r="J70" t="s">
+        <v>472</v>
+      </c>
       <c r="K70" t="s">
         <v>465</v>
       </c>
@@ -3479,6 +3689,9 @@
       <c r="E71" t="s">
         <v>313</v>
       </c>
+      <c r="J71" t="s">
+        <v>472</v>
+      </c>
       <c r="K71" t="s">
         <v>468</v>
       </c>
@@ -3502,6 +3715,9 @@
       <c r="E72" t="s">
         <v>314</v>
       </c>
+      <c r="J72" t="s">
+        <v>472</v>
+      </c>
       <c r="K72" t="s">
         <v>467</v>
       </c>
@@ -3525,6 +3741,9 @@
       <c r="E73" t="s">
         <v>315</v>
       </c>
+      <c r="J73" t="s">
+        <v>472</v>
+      </c>
       <c r="K73" t="s">
         <v>465</v>
       </c>
@@ -3545,6 +3764,9 @@
       <c r="E74" t="s">
         <v>316</v>
       </c>
+      <c r="J74" t="s">
+        <v>472</v>
+      </c>
       <c r="K74" t="s">
         <v>465</v>
       </c>
@@ -3568,6 +3790,9 @@
       <c r="E75" t="s">
         <v>317</v>
       </c>
+      <c r="J75" t="s">
+        <v>472</v>
+      </c>
       <c r="K75" t="s">
         <v>465</v>
       </c>
@@ -3591,6 +3816,9 @@
       <c r="E76" t="s">
         <v>319</v>
       </c>
+      <c r="J76" t="s">
+        <v>472</v>
+      </c>
       <c r="K76" t="s">
         <v>467</v>
       </c>
@@ -3614,6 +3842,9 @@
       <c r="E77" t="s">
         <v>321</v>
       </c>
+      <c r="J77" t="s">
+        <v>472</v>
+      </c>
       <c r="K77" t="s">
         <v>465</v>
       </c>
@@ -3637,6 +3868,9 @@
       <c r="E78" t="s">
         <v>322</v>
       </c>
+      <c r="J78" t="s">
+        <v>472</v>
+      </c>
       <c r="K78" t="s">
         <v>465</v>
       </c>
@@ -3660,6 +3894,9 @@
       <c r="E79" t="s">
         <v>323</v>
       </c>
+      <c r="J79" t="s">
+        <v>472</v>
+      </c>
       <c r="K79" t="s">
         <v>465</v>
       </c>
@@ -3683,6 +3920,9 @@
       <c r="E80" t="s">
         <v>324</v>
       </c>
+      <c r="J80" t="s">
+        <v>472</v>
+      </c>
       <c r="K80" t="s">
         <v>467</v>
       </c>
@@ -3706,6 +3946,9 @@
       <c r="E81" t="s">
         <v>326</v>
       </c>
+      <c r="J81" t="s">
+        <v>472</v>
+      </c>
       <c r="K81" t="s">
         <v>467</v>
       </c>
@@ -3729,6 +3972,9 @@
       <c r="E82" t="s">
         <v>327</v>
       </c>
+      <c r="J82" t="s">
+        <v>472</v>
+      </c>
       <c r="K82" t="s">
         <v>465</v>
       </c>
@@ -3752,6 +3998,9 @@
       <c r="E83" t="s">
         <v>329</v>
       </c>
+      <c r="J83" t="s">
+        <v>472</v>
+      </c>
       <c r="K83" t="s">
         <v>465</v>
       </c>
@@ -3775,6 +4024,9 @@
       <c r="E84" t="s">
         <v>330</v>
       </c>
+      <c r="J84" t="s">
+        <v>472</v>
+      </c>
       <c r="K84" t="s">
         <v>468</v>
       </c>
@@ -3798,6 +4050,9 @@
       <c r="E85" t="s">
         <v>332</v>
       </c>
+      <c r="J85" t="s">
+        <v>472</v>
+      </c>
       <c r="K85" t="s">
         <v>467</v>
       </c>
@@ -3821,6 +4076,9 @@
       <c r="E86" t="s">
         <v>335</v>
       </c>
+      <c r="J86" t="s">
+        <v>472</v>
+      </c>
       <c r="K86" t="s">
         <v>465</v>
       </c>
@@ -3844,6 +4102,9 @@
       <c r="E87" t="s">
         <v>336</v>
       </c>
+      <c r="J87" t="s">
+        <v>472</v>
+      </c>
       <c r="K87" t="s">
         <v>465</v>
       </c>
@@ -3867,6 +4128,9 @@
       <c r="E88" t="s">
         <v>337</v>
       </c>
+      <c r="J88" t="s">
+        <v>472</v>
+      </c>
       <c r="K88" t="s">
         <v>465</v>
       </c>
@@ -3890,6 +4154,9 @@
       <c r="E89" t="s">
         <v>338</v>
       </c>
+      <c r="J89" t="s">
+        <v>472</v>
+      </c>
       <c r="K89" t="s">
         <v>465</v>
       </c>
@@ -3913,6 +4180,9 @@
       <c r="E90" t="s">
         <v>341</v>
       </c>
+      <c r="J90" t="s">
+        <v>472</v>
+      </c>
       <c r="K90" t="s">
         <v>465</v>
       </c>
@@ -3936,6 +4206,9 @@
       <c r="E91" t="s">
         <v>342</v>
       </c>
+      <c r="J91" t="s">
+        <v>472</v>
+      </c>
       <c r="K91" t="s">
         <v>465</v>
       </c>
@@ -3959,6 +4232,9 @@
       <c r="E92" t="s">
         <v>343</v>
       </c>
+      <c r="J92" t="s">
+        <v>472</v>
+      </c>
       <c r="K92" t="s">
         <v>465</v>
       </c>
@@ -3982,6 +4258,9 @@
       <c r="E93" t="s">
         <v>345</v>
       </c>
+      <c r="J93" t="s">
+        <v>472</v>
+      </c>
       <c r="K93" t="s">
         <v>465</v>
       </c>
@@ -4005,6 +4284,9 @@
       <c r="E94" t="s">
         <v>346</v>
       </c>
+      <c r="J94" t="s">
+        <v>472</v>
+      </c>
       <c r="K94" t="s">
         <v>465</v>
       </c>
@@ -4028,6 +4310,9 @@
       <c r="E95" t="s">
         <v>347</v>
       </c>
+      <c r="J95" t="s">
+        <v>472</v>
+      </c>
       <c r="K95" t="s">
         <v>465</v>
       </c>
@@ -4051,6 +4336,9 @@
       <c r="E96" t="s">
         <v>350</v>
       </c>
+      <c r="J96" t="s">
+        <v>472</v>
+      </c>
       <c r="K96" t="s">
         <v>465</v>
       </c>
@@ -4074,6 +4362,9 @@
       <c r="E97" t="s">
         <v>352</v>
       </c>
+      <c r="J97" t="s">
+        <v>472</v>
+      </c>
       <c r="K97" t="s">
         <v>465</v>
       </c>
@@ -4097,6 +4388,9 @@
       <c r="E98" t="s">
         <v>353</v>
       </c>
+      <c r="J98" t="s">
+        <v>472</v>
+      </c>
       <c r="K98" t="s">
         <v>467</v>
       </c>
@@ -4120,6 +4414,9 @@
       <c r="E99" t="s">
         <v>355</v>
       </c>
+      <c r="J99" t="s">
+        <v>472</v>
+      </c>
       <c r="K99" t="s">
         <v>465</v>
       </c>
@@ -4143,6 +4440,9 @@
       <c r="E100" t="s">
         <v>356</v>
       </c>
+      <c r="J100" t="s">
+        <v>472</v>
+      </c>
       <c r="K100" t="s">
         <v>465</v>
       </c>
@@ -4166,6 +4466,9 @@
       <c r="E101" t="s">
         <v>358</v>
       </c>
+      <c r="J101" t="s">
+        <v>472</v>
+      </c>
       <c r="K101" t="s">
         <v>465</v>
       </c>
@@ -4189,6 +4492,9 @@
       <c r="E102" t="s">
         <v>359</v>
       </c>
+      <c r="J102" t="s">
+        <v>472</v>
+      </c>
       <c r="K102" t="s">
         <v>467</v>
       </c>
@@ -4212,6 +4518,9 @@
       <c r="E103" t="s">
         <v>360</v>
       </c>
+      <c r="J103" t="s">
+        <v>472</v>
+      </c>
       <c r="K103" t="s">
         <v>465</v>
       </c>
@@ -4235,6 +4544,9 @@
       <c r="E104" t="s">
         <v>361</v>
       </c>
+      <c r="J104" t="s">
+        <v>472</v>
+      </c>
       <c r="K104" t="s">
         <v>465</v>
       </c>
@@ -4258,6 +4570,9 @@
       <c r="E105" t="s">
         <v>362</v>
       </c>
+      <c r="J105" t="s">
+        <v>472</v>
+      </c>
       <c r="K105" t="s">
         <v>465</v>
       </c>
@@ -4281,6 +4596,9 @@
       <c r="E106" t="s">
         <v>363</v>
       </c>
+      <c r="J106" t="s">
+        <v>472</v>
+      </c>
       <c r="K106" t="s">
         <v>465</v>
       </c>
@@ -4304,6 +4622,9 @@
       <c r="E107" t="s">
         <v>364</v>
       </c>
+      <c r="J107" t="s">
+        <v>472</v>
+      </c>
       <c r="K107" t="s">
         <v>465</v>
       </c>
@@ -4327,6 +4648,9 @@
       <c r="E108" t="s">
         <v>365</v>
       </c>
+      <c r="J108" t="s">
+        <v>472</v>
+      </c>
       <c r="K108" t="s">
         <v>465</v>
       </c>
@@ -4350,6 +4674,9 @@
       <c r="E109" t="s">
         <v>366</v>
       </c>
+      <c r="J109" t="s">
+        <v>472</v>
+      </c>
       <c r="K109" t="s">
         <v>465</v>
       </c>
@@ -4373,6 +4700,9 @@
       <c r="E110" t="s">
         <v>368</v>
       </c>
+      <c r="J110" t="s">
+        <v>472</v>
+      </c>
       <c r="K110" t="s">
         <v>469</v>
       </c>
@@ -4396,6 +4726,9 @@
       <c r="E111" t="s">
         <v>370</v>
       </c>
+      <c r="J111" t="s">
+        <v>472</v>
+      </c>
       <c r="K111" t="s">
         <v>465</v>
       </c>
@@ -4419,6 +4752,9 @@
       <c r="E112" t="s">
         <v>372</v>
       </c>
+      <c r="J112" t="s">
+        <v>472</v>
+      </c>
       <c r="K112" t="s">
         <v>465</v>
       </c>
@@ -4442,6 +4778,9 @@
       <c r="E113" t="s">
         <v>373</v>
       </c>
+      <c r="J113" t="s">
+        <v>472</v>
+      </c>
       <c r="K113" t="s">
         <v>465</v>
       </c>
@@ -4465,6 +4804,9 @@
       <c r="E114" t="s">
         <v>375</v>
       </c>
+      <c r="J114" t="s">
+        <v>472</v>
+      </c>
       <c r="K114" t="s">
         <v>465</v>
       </c>
@@ -4488,6 +4830,9 @@
       <c r="E115" t="s">
         <v>376</v>
       </c>
+      <c r="J115" t="s">
+        <v>472</v>
+      </c>
       <c r="K115" t="s">
         <v>465</v>
       </c>
@@ -4511,6 +4856,9 @@
       <c r="E116" t="s">
         <v>377</v>
       </c>
+      <c r="J116" t="s">
+        <v>472</v>
+      </c>
       <c r="K116" t="s">
         <v>465</v>
       </c>
@@ -4534,6 +4882,9 @@
       <c r="E117" t="s">
         <v>378</v>
       </c>
+      <c r="J117" t="s">
+        <v>472</v>
+      </c>
       <c r="K117" t="s">
         <v>465</v>
       </c>
@@ -4557,6 +4908,9 @@
       <c r="E118" t="s">
         <v>379</v>
       </c>
+      <c r="J118" t="s">
+        <v>472</v>
+      </c>
       <c r="K118" t="s">
         <v>467</v>
       </c>
@@ -4580,6 +4934,9 @@
       <c r="E119" t="s">
         <v>380</v>
       </c>
+      <c r="J119" t="s">
+        <v>472</v>
+      </c>
       <c r="K119" t="s">
         <v>465</v>
       </c>
@@ -4603,6 +4960,9 @@
       <c r="E120" t="s">
         <v>381</v>
       </c>
+      <c r="J120" t="s">
+        <v>472</v>
+      </c>
       <c r="K120" t="s">
         <v>466</v>
       </c>
@@ -4626,6 +4986,9 @@
       <c r="E121" t="s">
         <v>383</v>
       </c>
+      <c r="J121" t="s">
+        <v>472</v>
+      </c>
       <c r="K121" t="s">
         <v>465</v>
       </c>
@@ -4649,6 +5012,9 @@
       <c r="E122" t="s">
         <v>384</v>
       </c>
+      <c r="J122" t="s">
+        <v>472</v>
+      </c>
       <c r="K122" t="s">
         <v>465</v>
       </c>
@@ -4669,6 +5035,9 @@
       <c r="E123" t="s">
         <v>386</v>
       </c>
+      <c r="J123" t="s">
+        <v>472</v>
+      </c>
       <c r="K123" t="s">
         <v>465</v>
       </c>
@@ -4692,6 +5061,9 @@
       <c r="E124" t="s">
         <v>387</v>
       </c>
+      <c r="J124" t="s">
+        <v>472</v>
+      </c>
       <c r="K124" t="s">
         <v>465</v>
       </c>
@@ -4715,6 +5087,9 @@
       <c r="E125" t="s">
         <v>388</v>
       </c>
+      <c r="J125" t="s">
+        <v>472</v>
+      </c>
       <c r="K125" t="s">
         <v>465</v>
       </c>
@@ -4738,6 +5113,9 @@
       <c r="E126" t="s">
         <v>390</v>
       </c>
+      <c r="J126" t="s">
+        <v>472</v>
+      </c>
       <c r="K126" t="s">
         <v>466</v>
       </c>
@@ -4761,6 +5139,9 @@
       <c r="E127" t="s">
         <v>391</v>
       </c>
+      <c r="J127" t="s">
+        <v>472</v>
+      </c>
       <c r="K127" t="s">
         <v>465</v>
       </c>
@@ -4784,6 +5165,9 @@
       <c r="E128" t="s">
         <v>392</v>
       </c>
+      <c r="J128" t="s">
+        <v>472</v>
+      </c>
       <c r="K128" t="s">
         <v>465</v>
       </c>
@@ -4807,6 +5191,9 @@
       <c r="E129" t="s">
         <v>394</v>
       </c>
+      <c r="J129" t="s">
+        <v>472</v>
+      </c>
       <c r="K129" t="s">
         <v>465</v>
       </c>
@@ -4830,6 +5217,9 @@
       <c r="E130" t="s">
         <v>395</v>
       </c>
+      <c r="J130" t="s">
+        <v>472</v>
+      </c>
       <c r="K130" t="s">
         <v>465</v>
       </c>
@@ -4853,6 +5243,9 @@
       <c r="E131" t="s">
         <v>329</v>
       </c>
+      <c r="J131" t="s">
+        <v>472</v>
+      </c>
       <c r="K131" t="s">
         <v>465</v>
       </c>
@@ -4876,6 +5269,9 @@
       <c r="E132" t="s">
         <v>397</v>
       </c>
+      <c r="J132" t="s">
+        <v>472</v>
+      </c>
       <c r="K132" t="s">
         <v>466</v>
       </c>
@@ -4899,6 +5295,9 @@
       <c r="E133" t="s">
         <v>399</v>
       </c>
+      <c r="J133" t="s">
+        <v>472</v>
+      </c>
       <c r="K133" t="s">
         <v>467</v>
       </c>
@@ -4922,6 +5321,9 @@
       <c r="E134" t="s">
         <v>400</v>
       </c>
+      <c r="J134" t="s">
+        <v>472</v>
+      </c>
       <c r="K134" t="s">
         <v>467</v>
       </c>
@@ -4945,6 +5347,9 @@
       <c r="E135" t="s">
         <v>402</v>
       </c>
+      <c r="J135" t="s">
+        <v>472</v>
+      </c>
       <c r="K135" t="s">
         <v>465</v>
       </c>
@@ -4968,6 +5373,9 @@
       <c r="E136" t="s">
         <v>403</v>
       </c>
+      <c r="J136" t="s">
+        <v>472</v>
+      </c>
       <c r="K136" t="s">
         <v>465</v>
       </c>
@@ -4991,6 +5399,9 @@
       <c r="E137" t="s">
         <v>405</v>
       </c>
+      <c r="J137" t="s">
+        <v>472</v>
+      </c>
       <c r="K137" t="s">
         <v>465</v>
       </c>
@@ -5014,6 +5425,9 @@
       <c r="E138" t="s">
         <v>407</v>
       </c>
+      <c r="J138" t="s">
+        <v>472</v>
+      </c>
       <c r="K138" t="s">
         <v>465</v>
       </c>
@@ -5037,6 +5451,9 @@
       <c r="E139" t="s">
         <v>408</v>
       </c>
+      <c r="J139" t="s">
+        <v>472</v>
+      </c>
       <c r="K139" t="s">
         <v>465</v>
       </c>
@@ -5060,6 +5477,9 @@
       <c r="E140" t="s">
         <v>409</v>
       </c>
+      <c r="J140" t="s">
+        <v>472</v>
+      </c>
       <c r="K140" t="s">
         <v>465</v>
       </c>
@@ -5083,6 +5503,9 @@
       <c r="E141" t="s">
         <v>411</v>
       </c>
+      <c r="J141" t="s">
+        <v>472</v>
+      </c>
       <c r="K141" t="s">
         <v>466</v>
       </c>
@@ -5106,6 +5529,9 @@
       <c r="E142" t="s">
         <v>412</v>
       </c>
+      <c r="J142" t="s">
+        <v>472</v>
+      </c>
       <c r="K142" t="s">
         <v>467</v>
       </c>
@@ -5126,6 +5552,9 @@
       <c r="E143" t="s">
         <v>413</v>
       </c>
+      <c r="J143" t="s">
+        <v>472</v>
+      </c>
       <c r="K143" t="s">
         <v>465</v>
       </c>
@@ -5149,6 +5578,9 @@
       <c r="E144" t="s">
         <v>414</v>
       </c>
+      <c r="J144" t="s">
+        <v>472</v>
+      </c>
       <c r="K144" t="s">
         <v>465</v>
       </c>
@@ -5172,6 +5604,9 @@
       <c r="E145" t="s">
         <v>415</v>
       </c>
+      <c r="J145" t="s">
+        <v>472</v>
+      </c>
       <c r="K145" t="s">
         <v>465</v>
       </c>
@@ -5195,6 +5630,9 @@
       <c r="E146" t="s">
         <v>416</v>
       </c>
+      <c r="J146" t="s">
+        <v>472</v>
+      </c>
       <c r="K146" t="s">
         <v>465</v>
       </c>
@@ -5218,6 +5656,9 @@
       <c r="E147" t="s">
         <v>417</v>
       </c>
+      <c r="J147" t="s">
+        <v>472</v>
+      </c>
       <c r="K147" t="s">
         <v>466</v>
       </c>
@@ -5241,6 +5682,9 @@
       <c r="E148" t="s">
         <v>418</v>
       </c>
+      <c r="J148" t="s">
+        <v>472</v>
+      </c>
       <c r="K148" t="s">
         <v>465</v>
       </c>
@@ -5264,6 +5708,9 @@
       <c r="E149" t="s">
         <v>419</v>
       </c>
+      <c r="J149" t="s">
+        <v>472</v>
+      </c>
       <c r="K149" t="s">
         <v>465</v>
       </c>
@@ -5287,6 +5734,9 @@
       <c r="E150" t="s">
         <v>420</v>
       </c>
+      <c r="J150" t="s">
+        <v>472</v>
+      </c>
       <c r="K150" t="s">
         <v>465</v>
       </c>
@@ -5310,6 +5760,9 @@
       <c r="E151" t="s">
         <v>421</v>
       </c>
+      <c r="J151" t="s">
+        <v>472</v>
+      </c>
       <c r="K151" t="s">
         <v>465</v>
       </c>
@@ -5333,6 +5786,9 @@
       <c r="E152" t="s">
         <v>422</v>
       </c>
+      <c r="J152" t="s">
+        <v>472</v>
+      </c>
       <c r="K152" t="s">
         <v>465</v>
       </c>
@@ -5356,6 +5812,9 @@
       <c r="E153" t="s">
         <v>423</v>
       </c>
+      <c r="J153" t="s">
+        <v>472</v>
+      </c>
       <c r="K153" t="s">
         <v>466</v>
       </c>
@@ -5379,6 +5838,9 @@
       <c r="E154" t="s">
         <v>424</v>
       </c>
+      <c r="J154" t="s">
+        <v>472</v>
+      </c>
       <c r="K154" t="s">
         <v>470</v>
       </c>
@@ -5402,6 +5864,9 @@
       <c r="E155" t="s">
         <v>425</v>
       </c>
+      <c r="J155" t="s">
+        <v>472</v>
+      </c>
       <c r="K155" t="s">
         <v>470</v>
       </c>
@@ -5425,6 +5890,9 @@
       <c r="E156" t="s">
         <v>426</v>
       </c>
+      <c r="J156" t="s">
+        <v>472</v>
+      </c>
       <c r="K156" t="s">
         <v>468</v>
       </c>
@@ -5448,6 +5916,9 @@
       <c r="E157" t="s">
         <v>427</v>
       </c>
+      <c r="J157" t="s">
+        <v>472</v>
+      </c>
       <c r="K157" t="s">
         <v>465</v>
       </c>
@@ -5471,6 +5942,9 @@
       <c r="E158" t="s">
         <v>428</v>
       </c>
+      <c r="J158" t="s">
+        <v>472</v>
+      </c>
       <c r="K158" t="s">
         <v>465</v>
       </c>
@@ -5494,6 +5968,9 @@
       <c r="E159" t="s">
         <v>429</v>
       </c>
+      <c r="J159" t="s">
+        <v>472</v>
+      </c>
       <c r="K159" t="s">
         <v>465</v>
       </c>
@@ -5517,6 +5994,9 @@
       <c r="E160" t="s">
         <v>430</v>
       </c>
+      <c r="J160" t="s">
+        <v>472</v>
+      </c>
       <c r="K160" t="s">
         <v>466</v>
       </c>
@@ -5540,6 +6020,9 @@
       <c r="E161" t="s">
         <v>432</v>
       </c>
+      <c r="J161" t="s">
+        <v>472</v>
+      </c>
       <c r="K161" t="s">
         <v>465</v>
       </c>
@@ -5563,6 +6046,9 @@
       <c r="E162" t="s">
         <v>433</v>
       </c>
+      <c r="J162" t="s">
+        <v>472</v>
+      </c>
       <c r="K162" t="s">
         <v>465</v>
       </c>
@@ -5586,6 +6072,9 @@
       <c r="E163" t="s">
         <v>434</v>
       </c>
+      <c r="J163" t="s">
+        <v>472</v>
+      </c>
       <c r="K163" t="s">
         <v>466</v>
       </c>
@@ -5609,6 +6098,9 @@
       <c r="E164" t="s">
         <v>435</v>
       </c>
+      <c r="J164" t="s">
+        <v>472</v>
+      </c>
       <c r="K164" t="s">
         <v>465</v>
       </c>
@@ -5632,6 +6124,9 @@
       <c r="E165" t="s">
         <v>436</v>
       </c>
+      <c r="J165" t="s">
+        <v>472</v>
+      </c>
       <c r="K165" t="s">
         <v>465</v>
       </c>
@@ -5655,6 +6150,9 @@
       <c r="E166" t="s">
         <v>438</v>
       </c>
+      <c r="J166" t="s">
+        <v>472</v>
+      </c>
       <c r="K166" t="s">
         <v>465</v>
       </c>
@@ -5674,6 +6172,9 @@
       </c>
       <c r="E167" t="s">
         <v>440</v>
+      </c>
+      <c r="J167" t="s">
+        <v>472</v>
       </c>
       <c r="K167" t="s">
         <v>465</v>
@@ -5698,6 +6199,9 @@
       <c r="E168" t="s">
         <v>441</v>
       </c>
+      <c r="J168" t="s">
+        <v>472</v>
+      </c>
       <c r="K168" t="s">
         <v>465</v>
       </c>
@@ -5721,6 +6225,9 @@
       <c r="E169" t="s">
         <v>342</v>
       </c>
+      <c r="J169" t="s">
+        <v>472</v>
+      </c>
       <c r="K169" t="s">
         <v>465</v>
       </c>
@@ -5744,6 +6251,9 @@
       <c r="E170" t="s">
         <v>442</v>
       </c>
+      <c r="J170" t="s">
+        <v>472</v>
+      </c>
       <c r="K170" t="s">
         <v>465</v>
       </c>
@@ -5767,6 +6277,9 @@
       <c r="E171" t="s">
         <v>443</v>
       </c>
+      <c r="J171" t="s">
+        <v>472</v>
+      </c>
       <c r="K171" t="s">
         <v>465</v>
       </c>
@@ -5790,6 +6303,9 @@
       <c r="E172" t="s">
         <v>445</v>
       </c>
+      <c r="J172" t="s">
+        <v>472</v>
+      </c>
       <c r="K172" t="s">
         <v>465</v>
       </c>
@@ -5813,6 +6329,9 @@
       <c r="E173" t="s">
         <v>446</v>
       </c>
+      <c r="J173" t="s">
+        <v>472</v>
+      </c>
       <c r="K173" t="s">
         <v>465</v>
       </c>
@@ -5836,6 +6355,9 @@
       <c r="E174" t="s">
         <v>447</v>
       </c>
+      <c r="J174" t="s">
+        <v>472</v>
+      </c>
       <c r="K174" t="s">
         <v>465</v>
       </c>
@@ -5859,6 +6381,9 @@
       <c r="E175" t="s">
         <v>448</v>
       </c>
+      <c r="J175" t="s">
+        <v>472</v>
+      </c>
       <c r="K175" t="s">
         <v>467</v>
       </c>
@@ -5882,6 +6407,9 @@
       <c r="E176" t="s">
         <v>449</v>
       </c>
+      <c r="J176" t="s">
+        <v>472</v>
+      </c>
       <c r="K176" t="s">
         <v>465</v>
       </c>
@@ -5905,6 +6433,9 @@
       <c r="E177" t="s">
         <v>451</v>
       </c>
+      <c r="J177" t="s">
+        <v>472</v>
+      </c>
       <c r="O177">
         <v>646920</v>
       </c>
@@ -5925,6 +6456,9 @@
       <c r="E178" t="s">
         <v>452</v>
       </c>
+      <c r="J178" t="s">
+        <v>472</v>
+      </c>
       <c r="K178" t="s">
         <v>465</v>
       </c>
@@ -5947,6 +6481,9 @@
       </c>
       <c r="E179" t="s">
         <v>454</v>
+      </c>
+      <c r="J179" t="s">
+        <v>472</v>
       </c>
       <c r="K179" t="s">
         <v>465</v>

</xml_diff>